<commit_message>
Rebuild the cicada IG on the docs site
Regenerated with the IG publisher and copied over. Adds everything the engine
gained this week: the forecast-reason, target-dose-status and data-integrity
code systems with their value sets, seven extensions
(target-dose-status-ext, evaluation-detail-ext and engine-version-ext on the
evaluation; series-group-ext, antigen-needing-dose-ext, doses-remaining-ext and
series-detail-ext on each recommendation), and a new page, "What Cicada
Returns", describing what each carries and why.

Built with -tx n/a. The first run sat in "Validating Resources" for 32 minutes
having used under four minutes of CPU, blocked on tx.fhir.org; the second
finished in two. The 147 QA errors are all java.net.SocketTimeoutException from
that same terminology validation, and none touches the new artifacts.

CLAUDE.md in this repo is modified by another session and is left alone.
</commit_message>
<xml_diff>
--- a/jaspr/web/cicada_ig/CodeSystem-EvalStatus.xlsx
+++ b/jaspr/web/cicada_ig/CodeSystem-EvalStatus.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
   <si>
     <t>Property</t>
   </si>
@@ -42,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Evaluation Status</t>
+    <t>Cicada Evaluation Status</t>
   </si>
   <si>
     <t>Status</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-11T14:37:07-05:00</t>
+    <t>2026-09-02T22:18:14-04:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>The status of the result of an evaluation.</t>
+    <t>Extension codes for dose evaluation status beyond the HL7 THO immunization-evaluation-dose-status CodeSystem. Only codes not covered by the standard are defined here.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -117,7 +117,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>4</t>
+    <t>1</t>
   </si>
   <si>
     <t>Level</t>
@@ -132,31 +132,13 @@
     <t>Definition</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>valid</t>
-  </si>
-  <si>
-    <t>Valid</t>
-  </si>
-  <si>
-    <t>not_valid</t>
-  </si>
-  <si>
-    <t>Not Valid</t>
-  </si>
-  <si>
     <t>extraneous</t>
   </si>
   <si>
     <t>Extraneous</t>
   </si>
   <si>
-    <t>sub_standard</t>
-  </si>
-  <si>
-    <t>Substandard</t>
+    <t>The dose was administered after the series was already complete. Every administered dose must be reported, so extraneous doses are tracked but do not affect the forecast.</t>
   </si>
 </sst>
 </file>
@@ -462,7 +444,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -481,58 +463,16 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="B2" t="s" s="2">
         <v>39</v>
       </c>
-      <c r="B2" t="s" s="2">
+      <c r="C2" t="s" s="2">
         <v>40</v>
-      </c>
-      <c r="C2" t="s" s="2">
-        <v>41</v>
       </c>
       <c r="D2" t="s" s="2">
         <v>41</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="2">
-        <v>39</v>
-      </c>
-      <c r="B3" t="s" s="2">
-        <v>42</v>
-      </c>
-      <c r="C3" t="s" s="2">
-        <v>43</v>
-      </c>
-      <c r="D3" t="s" s="2">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="2">
-        <v>39</v>
-      </c>
-      <c r="B4" t="s" s="2">
-        <v>44</v>
-      </c>
-      <c r="C4" t="s" s="2">
-        <v>45</v>
-      </c>
-      <c r="D4" t="s" s="2">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="2">
-        <v>39</v>
-      </c>
-      <c r="B5" t="s" s="2">
-        <v>46</v>
-      </c>
-      <c r="C5" t="s" s="2">
-        <v>47</v>
-      </c>
-      <c r="D5" t="s" s="2">
-        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>